<commit_message>
Update database monitoring air via Web App
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,6 +544,54 @@
       </c>
       <c r="P2" t="n">
         <v>1.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>WTM-5FCB9</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1342</v>
+      </c>
+      <c r="E3" t="n">
+        <v>333</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H3" t="n">
+        <v>243</v>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>141</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" t="n">
+        <v>5</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>